<commit_message>
Englisch: zweite Gegenlese-Runde – 53 geprüfte Vorschläge in Hilfe, Zimmer-Symbolen und Check-in-Blatt übernommen
Verworfen: verrutschte Zeilen der Rezeption, bereits abgelehnte „schedule“-Formulierungen
im Gästeportal, Kürzungen mit Inhaltsverlust und Begriffe, die von der Oberfläche
abweichen („demo“, „guided tour“, „routine cleaning“, „housekeeping board“ für die Anfragen).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sessions/Uebersetzung-alle-Texte-en-2026-10-17.xlsx
+++ b/Sessions/Uebersetzung-alle-Texte-en-2026-10-17.xlsx
@@ -37933,7 +37933,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>The overview is the front desk screen: all rooms by floor, the state of each room at a glance, and one click opens the dialog with check-in, check-out, PIN, check-in sheet, departure date, priority and history.</t>
+          <t>The overview is the front desk screen. It shows all rooms grouped by floor, with each room’s status at a glance. Clicking a room opens a dialog with check-in, check-out, PIN, check-in sheet, departure date, priority, and history.</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr"/>
@@ -38542,7 +38542,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>For complaints and special cases — manually; there’s nothing automatic. The room moves up on the housekeeping board, and the floor shows a purple warning light there. The priority ends on its own when the cleaning is finished.</t>
+          <t>For complaints and special cases, set a priority manually; it is never set automatically. The room moves up on the housekeeping board, and the floor is marked with a purple warning light. The priority clears automatically when cleaning is completed.</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr"/>
@@ -38658,7 +38658,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>In the room’s history: the “Check-out” entry carries the link. The statement is explicitly not an invoice — no guest name, no invoice number, no tax breakdown. It shows what’s to be collected.</t>
+          <t>In the room’s history, the “Check-out” entry links to the statement. This is not an invoice: it contains no guest name, invoice number, or tax breakdown. It shows the amount to be collected.</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr"/>
@@ -38774,7 +38774,7 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Cleaning only applies from that time — either the guest chose “not before” in the portal, or told the housekeeper at the door “later, please”. Which it was is shown in the room history. Until that time, the room isn’t open on either board; afterwards it is again on its own. How long guests may postpone in the portal is set under Property &amp; rules.</t>
+          <t>Cleaning becomes available at that time. Either the guest selected “not before” in the portal or asked the housekeeper at the door to come back later. The room’s history shows which. Until then, the room isn’t available for cleaning on either board; it opens automatically at the specified time. How long guests may postpone in the portal is set under Property &amp; rules.</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr"/>
@@ -39673,7 +39673,7 @@
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>The last 20 are listed, collapsed, below the open ones. Beyond that, you’ll find every request in the room’s history (30 days) and, if paid, on the statement of the stay.</t>
+          <t>The 20 most recent requests appear collapsed below the open requests. Beyond that, every request remains available in the room’s history for 30 days and, if it carried a price, on the stay statement.</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr"/>
@@ -40195,7 +40195,7 @@
       </c>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>Out of service is the recommended way for renovation and closure: no check-in, not on the housekeeping board, not on the room signs — but everything is kept, and one click brings the room back. The number stays taken. Deleting is permanent and frees the number.</t>
+          <t>For renovations or temporary closures, we recommend marking the room “Out of service”: it can’t be checked into, doesn’t appear on the housekeeping board or room signs, and all its history is retained. One click restores it to service, and the room number remains reserved. Deleting a room is permanent and frees the room number.</t>
         </is>
       </c>
       <c r="F82" s="7" t="inlineStr"/>
@@ -41558,7 +41558,7 @@
       </c>
       <c r="E129" s="6" t="inlineStr">
         <is>
-          <t>Two ways into the guest portal, chosen per property. With the fixed room QR, a code printed once is in the room, and every stay gets its PIN. With personal access, every stay gets its own code or link without a PIN, which expires at check-out.</t>
+          <t>There are two ways to access the guest portal, chosen for each property. With a fixed room QR code, a code is printed once and placed in the room, and each stay gets its own PIN. With personal access, each stay gets its own code or link, with no PIN; it expires at check-out.</t>
         </is>
       </c>
       <c r="F129" s="7" t="inlineStr"/>
@@ -41645,7 +41645,7 @@
       </c>
       <c r="E132" s="6" t="inlineStr">
         <is>
-          <t>Fixed QR + PIN if you can place or mount a sign in the rooms and want two factors (code in the room, PIN from the desk). Personal access if signs aren’t possible or wanted — more convenient for the guest, but anyone who sees the sheet has access. The page compares both in detail.</t>
+          <t>Choose fixed QR code + PIN if you can display a sign in each room and want two-factor access (the code in the room and the PIN from the front desk). Choose personal access if signs aren’t practical or desired. It’s more convenient for guests, but anyone who sees the sheet can access the portal for that stay. The page compares both in detail.</t>
         </is>
       </c>
       <c r="F132" s="7" t="inlineStr"/>
@@ -42138,7 +42138,7 @@
       </c>
       <c r="E149" s="6" t="inlineStr">
         <is>
-          <t>Three printouts are created in three places: the room sign per room (under Guest access or “Room signs”), the check-in sheet per stay (in the room dialog after check-in) and the access card per housekeeper (under Staff).</t>
+          <t>Three types of printouts are created in different places: a room sign for each room (under Guest access or “Room signs”), a check-in sheet for each stay (in the room dialog after check-in), and an access card for each housekeeper (under Staff).</t>
         </is>
       </c>
       <c r="F149" s="7" t="inlineStr"/>
@@ -42341,7 +42341,7 @@
       </c>
       <c r="E156" s="6" t="inlineStr">
         <is>
-          <t>Browsers don’t print background areas by default. The sheets are therefore built so that color only sits on lines and light tints with dark text — they work in grayscale too. If you want color, enable “Background graphics” in the print dialog.</t>
+          <t>Browsers don’t print background colors by default. The sheets are designed so that color appears only in lines and light shading with dark text, so they remain legible in grayscale. To print in color, enable “Background graphics” in the print dialog.</t>
         </is>
       </c>
       <c r="F156" s="7" t="inlineStr"/>
@@ -42399,7 +42399,7 @@
       </c>
       <c r="E158" s="6" t="inlineStr">
         <is>
-          <t>“Renew code” creates a new code for exactly this room; the old sign stops working from then on. Only the owner and managers can do this, and it always affects just one room. Print it again afterwards.</t>
+          <t>“Renew code” creates a new code for that room, invalidating the old room sign. Only the owner and managers can do this, and it affects just one room. Print the new sign afterward.</t>
         </is>
       </c>
       <c r="F158" s="7" t="inlineStr"/>
@@ -44313,7 +44313,7 @@
       </c>
       <c r="E224" s="6" t="inlineStr">
         <is>
-          <t>A tile in the guest portal that opens an outside website — such as the tipping app for the housekeeping team, a food delivery service or a taxi. A link doesn’t create a request: nothing on the board, nothing on the statement. Templates prefill the form; you adapt the address to your account or your city. The portal embeds nothing, it only links — the provider is responsible for the destination.</t>
+          <t>A tile in the guest portal that links to an external website, such as a tipping app for the housekeeping team, a food delivery service, or a taxi service. A link doesn’t create a request, so nothing appears on the Requests page or the stay statement. Templates prefill the form; adjust the address to your account or city. The portal only links to the external service; the provider is responsible for its content.</t>
         </is>
       </c>
       <c r="F224" s="7" t="inlineStr"/>
@@ -45096,7 +45096,7 @@
       </c>
       <c r="E251" s="6" t="inlineStr">
         <is>
-          <t>A recommendation, not an assignment: first a floor with an open priority, otherwise the one with the highest open urgency divided by the housekeepers there plus one. Departures weigh more the closer check-in gets. In a tie, the lower floor, so it doesn’t jump.</t>
+          <t>A recommendation, not an assignment: first choose a floor with an open priority; otherwise, choose the floor with the highest open urgency divided by the number of housekeepers there plus one. Departures carry more weight as check-in approaches. If there’s a tie, the lower floor is suggested to avoid the recommendation jumping back and forth.</t>
         </is>
       </c>
       <c r="F251" s="7" t="inlineStr"/>
@@ -45676,7 +45676,7 @@
       </c>
       <c r="E271" s="6" t="inlineStr">
         <is>
-          <t>After every room, the board recalculates. It suggests a switch if a prioritized room is open elsewhere, or if another floor weighs clearly more than the rest of the current one — usually because departures are waiting there and check-in is getting closer. On quiet days this rarely happens. The housekeeper decides: the switch is a slider; whoever stays simply carries on.</t>
+          <t>After each room, the board recalculates. It suggests switching floors if a room with an open priority is elsewhere, or if another floor’s workload is clearly higher than the current floor’s — usually because departures are waiting there and check-in is approaching. This is rare on quiet days. The housekeeper decides whether to switch; the switch control is a slider, and anyone who stays on the current floor can simply continue working.</t>
         </is>
       </c>
       <c r="F271" s="7" t="inlineStr"/>
@@ -46314,7 +46314,7 @@
       </c>
       <c r="E293" s="6" t="inlineStr">
         <is>
-          <t>The room immediately appears as open on the housekeeping board and in your overview. No appointment — housekeeping comes when it fits into the round. Tapping again withdraws the request. With “not before”, the guest chooses a full hour; until then the room isn’t open.</t>
+          <t>The room immediately appears as open on the housekeeping board and in your overview. There’s no appointment; housekeeping will get to it as part of their rounds. Tapping again withdraws the request. With “not before,” the guest selects a full hour, and the room won’t be available for cleaning until then.</t>
         </is>
       </c>
       <c r="F293" s="7" t="inlineStr"/>
@@ -46865,7 +46865,7 @@
       </c>
       <c r="E312" s="6" t="inlineStr">
         <is>
-          <t>Everything here is calculated, nothing stored: the basis is the housekeepers’ entries (shift start and end, breaks, other cleaning, start and finish per room) plus guest taps and check-outs. The period is in the address — a state can be linked and printed.</t>
+          <t>Everything here is calculated, not stored. It’s based on housekeepers’ entries (shift start and end, breaks, other cleaning, and start and finish times for each room), plus guest taps and check-outs. The selected period appears in the web address, so you can share or print a snapshot.</t>
         </is>
       </c>
       <c r="F312" s="7" t="inlineStr"/>
@@ -46923,7 +46923,7 @@
       </c>
       <c r="E314" s="6" t="inlineStr">
         <is>
-          <t>Net = shift without breaks. Remaining time = net minus room cleaning minus other cleaning — that is, walking, setup, waiting. A high remaining time usually means long walks or idle time between requests.</t>
+          <t>Net work time = shift time minus breaks. Remaining time = net work time minus room cleaning and other cleaning — in other words, time spent walking, setting up, or waiting. A high remaining-time figure usually points to long walks or idle time between requests.</t>
         </is>
       </c>
       <c r="F314" s="7" t="inlineStr"/>
@@ -47039,7 +47039,7 @@
       </c>
       <c r="E318" s="6" t="inlineStr">
         <is>
-          <t>Because the work record survives leaving. Anyone whose access has ended stays visible for their period. Only permanent deletion removes the entries — which is why it’s safeguarded by typing the name.</t>
+          <t>Because work records remain after someone leaves. Anyone whose access has ended remains visible for the period they worked. Only permanent deletion removes their entries, which is why deletion requires typing the name.</t>
         </is>
       </c>
       <c r="F318" s="7" t="inlineStr"/>
@@ -47097,7 +47097,7 @@
       </c>
       <c r="E320" s="6" t="inlineStr">
         <is>
-          <t>It writes a cleaning entry so daily cleaning counts as done — but the “per housekeeper” table shows housekeepers only. If cleanings are regularly marked as done at the desk, be aware that the reports don’t attribute these cleanings to any housekeeper.</t>
+          <t>It creates a cleaning record so the daily cleaning counts as completed. However, the “Per housekeeper” table includes only housekeepers. If front desk staff regularly mark cleanings as complete, those cleanings won’t be attributed to any housekeeper in the reports.</t>
         </is>
       </c>
       <c r="F320" s="7" t="inlineStr"/>
@@ -47155,7 +47155,7 @@
       </c>
       <c r="E322" s="6" t="inlineStr">
         <is>
-          <t>The property has chosen “Housekeeping activities: team only” under Property &amp; rules. Then there’s only the property total as a sum over the shifts; entries no longer carry a person after the shift ends. Switching back only works going forward — what’s anonymized stays anonymized.</t>
+          <t>Under Property &amp; rules, the property has selected “Housekeeping activities: team only.” Reports then show only the property-wide total across shifts, and entries are no longer linked to an individual after the shift ends. Switching back applies only going forward; anonymized entries stay anonymous.</t>
         </is>
       </c>
       <c r="F322" s="7" t="inlineStr"/>
@@ -47503,7 +47503,7 @@
       </c>
       <c r="E334" s="6" t="inlineStr">
         <is>
-          <t>In the portal header, in the room history at check-in and check-out, on completed requests and in the staff list. It’s changed everywhere at once.</t>
+          <t>It appears in the portal header, the room history at check-in and check-out, completed requests, and the staff list. The change takes effect everywhere at once.</t>
         </is>
       </c>
       <c r="F334" s="7" t="inlineStr"/>
@@ -47735,7 +47735,7 @@
       </c>
       <c r="E342" s="6" t="inlineStr">
         <is>
-          <t>Everything except the address: password, roles in all properties, display name and history. For the owner, invoices go to the new address from then on; billing details, payment method and plan stay unchanged.</t>
+          <t>Everything except the email address stays the same: password, roles across all properties, display name, and history. For the owner, invoices will go to the new address; billing details, payment method, and plan remain unchanged.</t>
         </is>
       </c>
       <c r="F342" s="7" t="inlineStr"/>
@@ -55448,7 +55448,7 @@
       </c>
       <c r="E631" s="6" t="inlineStr">
         <is>
-          <t>For every area there’s an explanation to look things up — symbols, questions, answers — and a guide: a guided tour over the real page that shows step by step what happens where. You can keep using the page as usual, nothing is locked; you can end the guide at any time with “End”. The “?” at the top right opens the explanation next to any page.</t>
+          <t>Each area has an explanation to look things up — symbols, questions, and answers — plus a guide: a guided tour of the actual page that shows you step by step how it works. You can continue using the page normally; nothing is locked. End the guide at any time with “End.” The “?” in the top-right corner opens the explanation beside any page.</t>
         </is>
       </c>
       <c r="F631" s="7" t="inlineStr"/>
@@ -55651,7 +55651,7 @@
       </c>
       <c r="E638" s="6" t="inlineStr">
         <is>
-          <t>Both take you to the page in question: the explanation in the sidebar next to it, the guide step by step on top of it — as often as you like.</t>
+          <t>Both take you to the relevant page: the explanation opens in the sidebar, while the guide walks you through the page step by step. You can use either as often as you like.</t>
         </is>
       </c>
       <c r="F638" s="7" t="inlineStr"/>
@@ -55854,7 +55854,7 @@
       </c>
       <c r="E645" s="6" t="inlineStr">
         <is>
-          <t>This is the board your housekeepers use on their phones. It’s a replica with example rooms — nothing is saved here and nobody is notified. Feel free to try everything; the guide restores the matching view for each step.</t>
+          <t>This is the board your housekeepers use on their phones. It’s a replica with sample rooms; nothing is saved and no one is notified. Feel free to try everything. The guide restores the appropriate view at each step.</t>
         </is>
       </c>
       <c r="F645" s="7" t="inlineStr"/>
@@ -55883,7 +55883,7 @@
       </c>
       <c r="E646" s="6" t="inlineStr">
         <is>
-          <t>Why a replica and not a tour of the real board? The housekeeping board has its own sign-in and its own session — it can’t be reached from the front desk. If you want to see the real thing, sign in at &lt;code&gt;{path}&lt;/code&gt; with a housekeeper’s account.</t>
+          <t>Why a replica instead of a tour of the live board? The housekeeping board has its own sign-in and session, so it can’t be accessed from the front desk. To see the live board, sign in at &lt;code&gt;{path}&lt;/code&gt; using a housekeeper’s account.</t>
         </is>
       </c>
       <c r="F646" s="7" t="inlineStr"/>
@@ -56144,7 +56144,7 @@
       </c>
       <c r="E655" s="6" t="inlineStr">
         <is>
-          <t>The guest portal as it looks on your guest’s phone. A replica with example values — property, room and services don’t come from your data, so the view shows something even before anything is set up. None of it is saved.</t>
+          <t>This is what the guest portal looks like on a guest’s phone. It’s a replica with sample data; the property, room, and services don’t come from your data, so the screen shows something even before setup is complete. Nothing is saved.</t>
         </is>
       </c>
       <c r="F655" s="7" t="inlineStr"/>
@@ -56173,7 +56173,7 @@
       </c>
       <c r="E656" s="6" t="inlineStr">
         <is>
-          <t>Your own texts differ in two places: which services appear is set in the service builder, and whether “not before” is offered at all — including the limit — is set under Property &amp; rules.</t>
+          <t>Your own text differs in two places: you configure which services appear in the service builder, and you set whether “Not before” is offered — including its cutoff time — under Property &amp; rules.</t>
         </is>
       </c>
       <c r="F656" s="7" t="inlineStr"/>
@@ -56700,7 +56700,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>The room accepts no check-in and appears on no housekeeping board. It keeps its history and can be put back into service under Rooms &amp; floors.</t>
+          <t>The room can’t be checked into and doesn’t appear on any housekeeping board. Its history is retained, and you can return it to service under Rooms &amp; floors.</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr"/>
@@ -56758,7 +56758,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>A stay is running. The guest has a PIN or a link and can request cleaning, set “Do not disturb” and request services in the portal.</t>
+          <t>A stay is in progress. The guest has a PIN or a link and can request cleaning, turn on “Do not disturb,” and request services in the portal.</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr"/>
@@ -56874,7 +56874,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>The guest set it in the portal. Nobody knocks, daily cleaning is skipped, and the room is grayed out on the housekeeping board. Only the guest can switch it off.</t>
+          <t>The guest enabled this in the portal. No one will knock, daily cleaning is skipped, and the room is grayed out on the housekeeping board. Only the guest can turn this setting off.</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr"/>
@@ -56932,7 +56932,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>One tap in the portal. The room immediately appears as open on the housekeeping board — no appointment; the housekeeping team comes when it fits into the round.</t>
+          <t>One tap in the portal makes the room appear as open on the housekeeping board, with no appointment. The housekeeping team will clean it when it fits into their rounds.</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr"/>
@@ -56990,7 +56990,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Not before a certain time: the guest chose this with the cleaning request, or told the housekeeper at the door “later, please”. Until then, the room counts as not open for all housekeepers; at that time it opens up again on its own.</t>
+          <t>The guest either selected a time in the cleaning request or asked the housekeeper at the door to come back later. Until then, the room isn’t available for cleaning to any housekeeper. It becomes available automatically at the specified time.</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr"/>
@@ -57048,7 +57048,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>The guest skips cleaning today — via the button in the portal or by telling the housekeeper at the door. Daily cleaning is skipped today and it doesn’t count as a cleaning; tomorrow it applies again. If the guest taps “Clean my room” after all, the room is open again immediately.</t>
+          <t>The guest skips cleaning for today, either by tapping the button in the portal or by telling the housekeeper at the door. Today’s daily cleaning is skipped and doesn’t count as a completed cleaning; daily cleaning resumes tomorrow. If the guest later taps “Clean my room,” the room becomes available immediately.</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr"/>
@@ -57106,7 +57106,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Only if the property cleans occupied rooms daily (Property &amp; rules): from the second night and from the set time — without a departure date no earlier than the check-out time —, as long as the room hasn’t been cleaned today and there’s no “Do not disturb”.</t>
+          <t>Only if the property cleans occupied rooms daily (under Property &amp; rules): cleaning becomes available from the second night, starting at the configured time. If no departure date is set, it won’t become available before the check-out time. This applies only if the room hasn’t been cleaned today and “Do not disturb” isn’t on.</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr"/>
@@ -57222,7 +57222,7 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Set manually by the front desk — for complaints and special cases. The room moves up on the housekeeping board and the floor shows a purple warning light. Never automatic.</t>
+          <t>Set manually by the front desk for complaints or special cases. The room moves up the housekeeping board, and the floor displays a purple warning light. This is never automatic.</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr"/>
@@ -57280,7 +57280,7 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>A housekeeper has pulled the start slider; their name appears in the room. If finishing is forgotten, the room reopens on its own after the time limit.</t>
+          <t>A housekeeper has moved the start slider, and their name appears in the room. If they forget to mark the cleaning complete, the room automatically reopens after the time limit.</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr"/>
@@ -57338,7 +57338,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>The guest requested something nobody has checked off yet. Requests are under “Requests” in the navigation; check them off there or in the room dialog.</t>
+          <t>The guest has made a request that hasn’t been marked complete. Requests appear under “Requests” in the navigation; mark them complete there or in the room dialog.</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr"/>
@@ -57396,7 +57396,7 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>At least one open request concerns a service marked “urgent” in the builder. Bell, ring and the number in the navigation flash red until it’s checked off.</t>
+          <t>At least one open request is for a service marked “urgent” in the service builder. The bell, ring, and navigation count flash red until the request is marked complete.</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr"/>
@@ -57454,7 +57454,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Beats everything else. As long as the priority stands, the bar is purple — even for a checked-out room.</t>
+          <t>Overrides all other states. As long as the priority is active, the bar stays purple — even after check-out.</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr"/>
@@ -57512,7 +57512,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Only on the housekeeping board: someone from the team is in the room right now. At the front desk, only the spinner shows this; the bar keeps its color.</t>
+          <t>Only on the housekeeping board: a team member is currently in the room. On the front desk screen, this is shown only by the spinner; the bar keeps its color.</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr"/>
@@ -57628,7 +57628,7 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>The guest tapped, or the property’s daily cleaning is due. A postponed request (“from HH:MM”) only colors the bar at that time.</t>
+          <t>The guest has requested cleaning, or the property’s daily cleaning is due. A postponed request (“from HH:MM”) changes the bar’s color only at the specified time.</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr"/>
@@ -57860,7 +57860,7 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Only on the housekeeping board: vacant, occupied without a request, “Do not disturb”, or a request that applies only later. Visible but grayed out — not blocked.</t>
+          <t>Only on the housekeeping board: vacant, occupied with no request, “Do not disturb,” or a request scheduled for later. The room remains visible but grayed out — it isn’t blocked.</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr"/>
@@ -58503,7 +58503,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Every cleaning that isn’t needed saves water, detergent and energy — it is your choice in the portal.</t>
+          <t>Every unnecessary cleaning saves water, detergent, and energy. You decide whether you need cleaning in the guest portal.</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr"/>
@@ -58706,7 +58706,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>The guest portal connects you to the front desk straight from your room — around the clock, without a phone call.</t>
+          <t>The guest portal lets you contact the front desk directly from your room, 24/7, without calling.</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr"/>
@@ -58764,7 +58764,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Ask for fresh towels, report a repair or request other services directly in the portal — the front desk sees your request immediately.</t>
+          <t>Request fresh towels, report a problem, or ask for other services directly in the portal. The front desk receives your request immediately.</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr"/>
@@ -58793,7 +58793,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Your room is cleaned daily from {due}, on your day of departure after check-out — you don’t have to request anything. Would you like an extra cleaning in between? Simply request it in the portal.</t>
+          <t>Your room is cleaned daily starting at {due}, and after check-out on your departure day — no request is needed. For an extra cleaning in between, tap “Clean my room” in the portal.</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr"/>
@@ -58822,7 +58822,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Your room is cleaned on request: please ask for cleaning in the portal whenever it suits you — without your request, nobody enters your room.</t>
+          <t>Your room is cleaned on request. Please request cleaning in the portal whenever it suits you. Without a request, no one will enter your room.</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr"/>
@@ -58880,7 +58880,7 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> You can also postpone cleaning until {limit} at the latest — no one will come before then.</t>
+          <t xml:space="preserve"> You can also postpone cleaning in the portal until {limit} at the latest. No one will come before then.</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr"/>
@@ -58909,7 +58909,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>No cleaning needed today? One tap on “{skip}” in the portal saves water, detergent and energy — cleaning resumes tomorrow.</t>
+          <t>Don’t need cleaning today? Tap “{skip}” in the portal to save water, detergent, and energy. Daily cleaning resumes tomorrow.</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr"/>
@@ -58938,7 +58938,7 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Less cleaning, less consumption: every cleaning that isn’t needed saves water, detergent and energy. That is why we only come when you want us to.</t>
+          <t>Less cleaning means lower resource use. Every unnecessary cleaning saves water, detergent, and energy, so we come only when you want us to.</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr"/>
@@ -58967,7 +58967,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>This access is personal and needs no PIN — please do not share it. It is valid for this stay only and expires at check-out.</t>
+          <t>This access is personal and doesn’t require a PIN. Please don’t share it. It’s valid only for this stay and expires at check-out.</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr"/>
@@ -59025,7 +59025,7 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Open the address, enter your room number and PIN — you stay signed in afterwards. The PIN is valid until check-out.</t>
+          <t>Open the web address, enter your room number and PIN, and you’ll stay signed in. The PIN is valid until check-out.</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Englisch einheitlich: Komma vor dem letzten Aufzählungsglied, Punkt und Komma in Anführungszeichen; zwei Übernahmen der ersten Gegenlese-Runde korrigiert
„scheduled“ in der Statuskarte versprach einen Termin, „individual access links“ wich von
„personal access“ ab. Wächter en-style.test.ts für die Anführungszeichen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sessions/Uebersetzung-alle-Texte-en-2026-10-17.xlsx
+++ b/Sessions/Uebersetzung-alle-Texte-en-2026-10-17.xlsx
@@ -1103,7 +1103,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>We use individual access links. Please scan the QR code on the sheet you received at check-in, or open the link in your email. Use the form below only if you received a PIN at check-in.</t>
+          <t>We use personal access links. Please scan the QR code on the sheet you received at check-in, or open the link in your email. Use the form below only if you received a PIN at check-in.</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr"/>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Cleaning is scheduled.</t>
+          <t>Cleaning is planned for today.</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr"/>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Housekeeping is scheduled to visit today.</t>
+          <t>Housekeeping will stop by today — there’s no fixed time.</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr"/>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>We clean daily. If you don’t need your room cleaned today, tap “No cleaning today”.</t>
+          <t>We clean daily. If you don’t need your room cleaned today, tap “No cleaning today.”</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr"/>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Would you like it cleaned again? Then tap “Clean my room”.</t>
+          <t>Would you like it cleaned again? Then tap “Clean my room.”</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr"/>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Thank you — that saves water and detergent. Changed your mind? Then tap “Clean my room”.</t>
+          <t>Thank you — that saves water and detergent. Changed your mind? Then tap “Clean my room.”</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr"/>
@@ -1799,7 +1799,7 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Your room will be cleaned after check-out. Would you like it cleaned before then? Tap “Clean my room”.</t>
+          <t>Your room will be cleaned after check-out. Would you like it cleaned before then? Tap “Clean my room.”</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr"/>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Starting tomorrow, we clean daily from {time}. Would you like your room cleaned today? Tap “Clean my room”.</t>
+          <t>Starting tomorrow, we clean daily from {time}. Would you like your room cleaned today? Tap “Clean my room.”</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr"/>
@@ -9697,7 +9697,7 @@
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>Still open and therefore not in the total. Already done? Then check it off now — check-out closes open requests as “not provided”.</t>
+          <t>Still open and therefore not in the total. Already done? Then check it off now — check-out closes open requests as “not provided.”</t>
         </is>
       </c>
       <c r="F89" s="7" t="inlineStr"/>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="E100" s="6" t="inlineStr">
         <is>
-          <t>One open request ({amount}) will be closed as “not provided”.</t>
+          <t>One open request ({amount}) will be closed as “not provided.”</t>
         </is>
       </c>
       <c r="F100" s="7" t="inlineStr"/>
@@ -10045,7 +10045,7 @@
       </c>
       <c r="E101" s="6" t="inlineStr">
         <is>
-          <t>{count} open requests ({amount}) will be closed as “not provided”.</t>
+          <t>{count} open requests ({amount}) will be closed as “not provided.”</t>
         </is>
       </c>
       <c r="F101" s="7" t="inlineStr"/>
@@ -12887,7 +12887,7 @@
       </c>
       <c r="E199" s="6" t="inlineStr">
         <is>
-          <t>Letters, digits, period, underscore and hyphen only</t>
+          <t>Letters, digits, period, underscore, and hyphen only</t>
         </is>
       </c>
       <c r="F199" s="7" t="inlineStr"/>
@@ -13061,7 +13061,7 @@
       </c>
       <c r="E205" s="6" t="inlineStr">
         <is>
-          <t>Housekeepers sign in with the &lt;b&gt;username&lt;/b&gt; and PIN — not the display name, which only appears on the board and the access card. The PIN (6 digits) and access card are created automatically — hand them over via “Print card”.</t>
+          <t>Housekeepers sign in with the &lt;b&gt;username&lt;/b&gt; and PIN — not the display name, which only appears on the board and the access card. The PIN (6 digits) and access card are created automatically — hand them over via “Print card.”</t>
         </is>
       </c>
       <c r="F205" s="7" t="inlineStr"/>
@@ -13235,7 +13235,7 @@
       </c>
       <c r="E211" s="6" t="inlineStr">
         <is>
-          <t>Front desk accounts handle day-to-day work (check-in/out, requests, printing) — settings, room setup and services remain with the owner and managers. The person receives an email invitation and sets their own password.</t>
+          <t>Front desk accounts handle day-to-day work (check-in/out, requests, printing) — settings, room setup, and services remain with the owner and managers. The person receives an email invitation and sets their own password.</t>
         </is>
       </c>
       <c r="F211" s="7" t="inlineStr"/>
@@ -14946,7 +14946,7 @@
       </c>
       <c r="E270" s="6" t="inlineStr">
         <is>
-          <t>{count} activity log entry{period} — shifts, breaks and cleanings disappear from the reports</t>
+          <t>{count} activity log entry{period} — shifts, breaks, and cleanings disappear from the reports</t>
         </is>
       </c>
       <c r="F270" s="7" t="inlineStr"/>
@@ -14975,7 +14975,7 @@
       </c>
       <c r="E271" s="6" t="inlineStr">
         <is>
-          <t>{count} activity log entries{period} — shifts, breaks and cleanings disappear from the reports</t>
+          <t>{count} activity log entries{period} — shifts, breaks, and cleanings disappear from the reports</t>
         </is>
       </c>
       <c r="F271" s="7" t="inlineStr"/>
@@ -16657,7 +16657,7 @@
       </c>
       <c r="E329" s="6" t="inlineStr">
         <is>
-          <t>This property evaluates cleaning &lt;b&gt;as a team only&lt;/b&gt; (setting under Property &amp; rules): the figures above are the total over {shifts} in this period; there’s no “per housekeeper” table and no daily log. When each room was cleaned is shown in the room history, where the person appears as “Housekeeping team”.</t>
+          <t>This property evaluates cleaning &lt;b&gt;as a team only&lt;/b&gt; (setting under Property &amp; rules): the figures above are the total over {shifts} in this period; there’s no “per housekeeper” table and no daily log. When each room was cleaned is shown in the room history, where the person appears as “Housekeeping team.”</t>
         </is>
       </c>
       <c r="F329" s="7" t="inlineStr"/>
@@ -19412,7 +19412,7 @@
       </c>
       <c r="E424" s="6" t="inlineStr">
         <is>
-          <t>An account already exists for this email address. If the person is already a manager in the account, choose them via “Add an existing manager”.</t>
+          <t>An account already exists for this email address. If the person is already a manager in the account, choose them via “Add an existing manager.”</t>
         </is>
       </c>
       <c r="F424" s="7" t="inlineStr"/>
@@ -20021,7 +20021,7 @@
       </c>
       <c r="E445" s="6" t="inlineStr">
         <is>
-          <t>Room numbers — single, comma list or range</t>
+          <t>Room numbers — single, comma list, or range</t>
         </is>
       </c>
       <c r="F445" s="7" t="inlineStr"/>
@@ -20050,7 +20050,7 @@
       </c>
       <c r="E446" s="6" t="inlineStr">
         <is>
-          <t>Room numbers per floor — single, comma list or range</t>
+          <t>Room numbers per floor — single, comma list, or range</t>
         </is>
       </c>
       <c r="F446" s="7" t="inlineStr"/>
@@ -20514,7 +20514,7 @@
       </c>
       <c r="E462" s="6" t="inlineStr">
         <is>
-          <t>Click a room, floor or building to &lt;b&gt;edit&lt;/b&gt; it, &lt;b&gt;take it out of service&lt;/b&gt; or &lt;b&gt;delete&lt;/b&gt; it. A typo? Editing changes number, floor and building without losing anything.</t>
+          <t>Click a room, floor, or building to &lt;b&gt;edit&lt;/b&gt; it, &lt;b&gt;take it out of service&lt;/b&gt;, or &lt;b&gt;delete&lt;/b&gt; it. A typo? Editing changes number, floor, and building without losing anything.</t>
         </is>
       </c>
       <c r="F462" s="7" t="inlineStr"/>
@@ -20920,7 +20920,7 @@
       </c>
       <c r="E476" s="6" t="inlineStr">
         <is>
-          <t>Correct number, floor or building — nothing is lost</t>
+          <t>Correct number, floor, or building — nothing is lost</t>
         </is>
       </c>
       <c r="F476" s="7" t="inlineStr"/>
@@ -23849,7 +23849,7 @@
       </c>
       <c r="E577" s="6" t="inlineStr">
         <is>
-          <t>A &lt;b&gt;maintenance report&lt;/b&gt; is meant for defects and repairs — something about the room, not the stay. Such requests stay open at check-out (a defect doesn’t disappear with the guest), appear on no check-out statement and show a warning at the next check-in.</t>
+          <t>A &lt;b&gt;maintenance report&lt;/b&gt; is meant for defects and repairs — something about the room, not the stay. Such requests stay open at check-out (a defect doesn’t disappear with the guest), appear on no check-out statement, and show a warning at the next check-in.</t>
         </is>
       </c>
       <c r="F577" s="7" t="inlineStr"/>
@@ -26082,7 +26082,7 @@
       </c>
       <c r="E654" s="6" t="inlineStr">
         <is>
-          <t>Change your sign-in address, display name and password</t>
+          <t>Change your sign-in address, display name, and password</t>
         </is>
       </c>
       <c r="F654" s="7" t="inlineStr"/>
@@ -26430,7 +26430,7 @@
       </c>
       <c r="E666" s="6" t="inlineStr">
         <is>
-          <t>Property address (lowercase letters, digits and hyphens only)</t>
+          <t>Property address (lowercase letters, digits, and hyphens only)</t>
         </is>
       </c>
       <c r="F666" s="7" t="inlineStr"/>
@@ -26604,7 +26604,7 @@
       </c>
       <c r="E672" s="6" t="inlineStr">
         <is>
-          <t>From the second day, guests see a request for a review at the bottom of the guest portal, and after check-out a thank-you page with this link. You can find your Google link in your Google Business Profile under “Get more reviews”. Tripadvisor, Booking.com, HolidayCheck or your own page work too. Leave empty if you don’t want to ask for reviews.</t>
+          <t>From the second day, guests see a request for a review at the bottom of the guest portal, and after check-out a thank-you page with this link. You can find your Google link in your Google Business Profile under “Get more reviews.” Tripadvisor, Booking.com, HolidayCheck, or your own page work too. Leave empty if you don’t want to ask for reviews.</t>
         </is>
       </c>
       <c r="F672" s="7" t="inlineStr"/>
@@ -26749,7 +26749,7 @@
       </c>
       <c r="E677" s="6" t="inlineStr">
         <is>
-          <t>If a cleaning was started but not finished, the room is open on the board again after this time. The history then shows “Cleaning not finished (time limit)”.</t>
+          <t>If a cleaning was started but not finished, the room is open on the board again after this time. The history then shows “Cleaning not finished (time limit).”</t>
         </is>
       </c>
       <c r="F677" s="7" t="inlineStr"/>
@@ -26807,7 +26807,7 @@
       </c>
       <c r="E679" s="6" t="inlineStr">
         <is>
-          <t>From the day after arrival, occupied rooms appear on the housekeeping board on their own at the chosen time, until they’ve been cleaned that day. Exceptions are “Do not disturb”, “No cleaning today” and the day of departure.</t>
+          <t>From the day after arrival, occupied rooms appear on the housekeeping board on their own at the chosen time, until they’ve been cleaned that day. Exceptions are “Do not disturb,” “No cleaning today” and the day of departure.</t>
         </is>
       </c>
       <c r="F679" s="7" t="inlineStr"/>
@@ -27271,7 +27271,7 @@
       </c>
       <c r="E695" s="6" t="inlineStr">
         <is>
-          <t>For countries and businesses where the work of individual housekeepers may not or should not be measured. The property still sees when each room was cleaned and how much the team does — but not who: no table per housekeeper, no daily log, and the room history shows “Housekeeping team”.</t>
+          <t>For countries and businesses where the work of individual housekeepers may not or should not be measured. The property still sees when each room was cleaned and how much the team does — but not who: no table per housekeeper, no daily log, and the room history shows “Housekeeping team.”</t>
         </is>
       </c>
       <c r="F695" s="7" t="inlineStr"/>
@@ -28460,7 +28460,7 @@
       </c>
       <c r="E736" s="6" t="inlineStr">
         <is>
-          <t>You don’t want QR codes in the rooms — for looks, heritage protection or frequent renovation.</t>
+          <t>You don’t want QR codes in the rooms — for looks, heritage protection, or frequent renovation.</t>
         </is>
       </c>
       <c r="F736" s="7" t="inlineStr"/>
@@ -29620,7 +29620,7 @@
       </c>
       <c r="E776" s="6" t="inlineStr">
         <is>
-          <t>Saved. The portals, the next printouts and emails follow the new choice.</t>
+          <t>Saved. The portals, the next printouts, and emails follow the new choice.</t>
         </is>
       </c>
       <c r="F776" s="7" t="inlineStr"/>
@@ -29794,7 +29794,7 @@
       </c>
       <c r="E782" s="6" t="inlineStr">
         <is>
-          <t>PNG, JPG or SVG, 1 MB max. On the sheet, it appears at the top left, at most 55 × 16 mm. A light logo meant for dark backgrounds is invisible on white paper — the preview on the left shows it as it will be printed.</t>
+          <t>PNG, JPG, or SVG, 1 MB max. On the sheet, it appears at the top left, at most 55 × 16 mm. A light logo meant for dark backgrounds is invisible on white paper — the preview on the left shows it as it will be printed.</t>
         </is>
       </c>
       <c r="F782" s="7" t="inlineStr"/>
@@ -30258,7 +30258,7 @@
       </c>
       <c r="E798" s="6" t="inlineStr">
         <is>
-          <t>A confirmation link is sent to the new address; only clicking it makes the switch. Until then, you keep signing in with your current address. Afterwards, the previous address receives a notice. Password, roles and history stay as they are.</t>
+          <t>A confirmation link is sent to the new address; only clicking it makes the switch. Until then, you keep signing in with your current address. Afterwards, the previous address receives a notice. Password, roles, and history stay as they are.</t>
         </is>
       </c>
       <c r="F798" s="7" t="inlineStr"/>
@@ -30287,7 +30287,7 @@
       </c>
       <c r="E799" s="6" t="inlineStr">
         <is>
-          <t>As the owner, you’ll receive invoices at the new address from then on. Billing details, payment method and plan stay unchanged.</t>
+          <t>As the owner, you’ll receive invoices at the new address from then on. Billing details, payment method, and plan stay unchanged.</t>
         </is>
       </c>
       <c r="F799" s="7" t="inlineStr"/>
@@ -30838,7 +30838,7 @@
       </c>
       <c r="E818" s="6" t="inlineStr">
         <is>
-          <t>This link is invalid, expired or has already been used. Request a new one under “My account”.</t>
+          <t>This link is invalid, expired, or has already been used. Request a new one under “My account.”</t>
         </is>
       </c>
       <c r="F818" s="7" t="inlineStr"/>
@@ -30896,7 +30896,7 @@
       </c>
       <c r="E820" s="6" t="inlineStr">
         <is>
-          <t>The switch failed. Please try again later or request a new link under “My account”.</t>
+          <t>The switch failed. Please try again later or request a new link under “My account.”</t>
         </is>
       </c>
       <c r="F820" s="7" t="inlineStr"/>
@@ -31679,7 +31679,7 @@
       </c>
       <c r="E847" s="6" t="inlineStr">
         <is>
-          <t>Check out all active stays, neutralize room states and delete open requests?</t>
+          <t>Check out all active stays, neutralize room states, and delete open requests?</t>
         </is>
       </c>
       <c r="F847" s="7" t="inlineStr"/>
@@ -31711,7 +31711,7 @@
       <c r="E848" s="6" t="inlineStr">
         <is>
           <t>Remove test data completely?
-This deletes ALL stays, requests, room histories and housekeeping entries of this property — including those not from a scenario. Rooms and staff remain.
+This deletes ALL stays, requests, room histories, and housekeeping entries of this property — including those not from a scenario. Rooms and staff remain.
 Afterwards, all rooms are without history again and can be deleted without data loss.</t>
         </is>
       </c>
@@ -32640,7 +32640,7 @@
       </c>
       <c r="E880" s="6" t="inlineStr">
         <is>
-          <t>Delete the property’s stays, requests, history and housekeeping entries</t>
+          <t>Delete the property’s stays, requests, history, and housekeeping entries</t>
         </is>
       </c>
       <c r="F880" s="7" t="inlineStr"/>
@@ -32843,7 +32843,7 @@
       </c>
       <c r="E887" s="6" t="inlineStr">
         <is>
-          <t>The address may only contain lowercase letters, digits and hyphens ({max} characters max., not starting or ending with a hyphen).</t>
+          <t>The address may only contain lowercase letters, digits, and hyphens ({max} characters max., not starting or ending with a hyphen).</t>
         </is>
       </c>
       <c r="F887" s="7" t="inlineStr"/>
@@ -35487,7 +35487,7 @@
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>Invitation link — hand it over via messenger, text message or note</t>
+          <t>Invitation link — hand it over via messenger, text message, or note</t>
         </is>
       </c>
       <c r="F61" s="7" t="inlineStr"/>
@@ -36681,7 +36681,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Print once, place in the room, hang it up or put it in the folder — the guest scans and only types the PIN they receive at check-in. The compact format can be cut apart. A new code makes the room’s old sign stop working.</t>
+          <t>Print once, place in the room, hang it up, or put it in the folder — the guest scans and only types the PIN they receive at check-in. The compact format can be cut apart. A new code makes the room’s old sign stop working.</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr"/>
@@ -37754,7 +37754,7 @@
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>This statement is &lt;b&gt;not an invoice&lt;/b&gt; and not a tax document. It lists only the extra services for this room ordered via the guest portal; accommodation, other items and invoicing are handled in the property’s own system.</t>
+          <t>This statement is &lt;b&gt;not an invoice&lt;/b&gt; and not a tax document. It lists only the extra services for this room ordered via the guest portal; accommodation, other items, and invoicing are handled in the property’s own system.</t>
         </is>
       </c>
       <c r="F62" s="7" t="inlineStr"/>
@@ -38078,7 +38078,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Several symbols at once are normal — occupied, cleaning requested and an open request, for example. The tile’s tooltip states everything in plain words.</t>
+          <t>Several symbols at once are normal — occupied, cleaning requested, and an open request, for example. The tile’s tooltip states everything in plain words.</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr"/>
@@ -38310,7 +38310,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>RoSe only shows what has actually been reported: check-out says “cleaning open”, and only a housekeeper finishing — or your “Mark cleaning as done” in the dialog — says “ready”. RoSe doesn’t guess whether someone has been there in the meantime.</t>
+          <t>RoSe only shows what has actually been reported: check-out says “cleaning open,” and only a housekeeper finishing — or your “Mark cleaning as done” in the dialog — says “ready.” RoSe doesn’t guess whether someone has been there in the meantime.</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr"/>
@@ -38484,7 +38484,7 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>No — the default is “open”, so check-in stays one click. If you enter it, daily cleaning is skipped on the day of departure and the tile shows the suitcase. You can add or extend it at any time in the dialog. An outdated date (yesterday) counts as unknown, so a forgotten update doesn’t switch off daily cleaning permanently.</t>
+          <t>No — the default is “open,” so check-in stays one click. If you enter it, daily cleaning is skipped on the day of departure and the tile shows the suitcase. You can add or extend it at any time in the dialog. An outdated date (yesterday) counts as unknown, so a forgotten update doesn’t switch off daily cleaning permanently.</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr"/>
@@ -38600,7 +38600,7 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>PIN, link and the guest’s session stop working immediately, and the room goes to “cleaning open”. Open service requests of this stay are closed as “not provided” — check off what was actually provided in the same box beforehand. Maintenance reports (defects) stay open. If the guest ordered something paid, the total appears in the dialog before you confirm.</t>
+          <t>PIN, link, and the guest’s session stop working immediately, and the room goes to “cleaning open.” Open service requests of this stay are closed as “not provided” — check off what was actually provided in the same box beforehand. Maintenance reports (defects) stay open. If the guest ordered something paid, the total appears in the dialog before you confirm.</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr"/>
@@ -38716,7 +38716,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>The room’s last 30 days: guest taps (always just “Guest”, never an identity), cleanings with names, check-in and check-out with the person at the desk, service requests. “Cleaning not finished (time limit)” appears there too — the history is the work record and the tool for complaints.</t>
+          <t>The room’s last 30 days: guest taps (always just “Guest,” never an identity), cleanings with names, check-in and check-out with the person at the desk, service requests. “Cleaning not finished (time limit)” appears there too — the history is the work record and the tool for complaints.</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr"/>
@@ -39499,7 +39499,7 @@
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>It isn’t gone, but closed as “not provided” and listed under “Recently closed”. Requests belong to the stay, not the room — otherwise tomorrow the board would show a request for an empty room.</t>
+          <t>It isn’t gone, but closed as “not provided” and listed under “Recently closed.” Requests belong to the stay, not the room — otherwise tomorrow the board would show a request for an empty room.</t>
         </is>
       </c>
       <c r="F58" s="7" t="inlineStr"/>
@@ -39528,7 +39528,7 @@
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>What’s a “maintenance report”, and why does it stay open?</t>
+          <t>What’s a “maintenance report,” and why does it stay open?</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr"/>
@@ -39731,7 +39731,7 @@
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>Check the room’s history to see whether a request arrived. The most common causes: the guest canceled before sending, or used a tile under “Useful links”, such as a food delivery service — that leads to an outside site and doesn’t create a request.</t>
+          <t>Check the room’s history to see whether a request arrived. The most common causes: the guest canceled before sending, or used a tile under “Useful links,” such as a food delivery service — that leads to an outside site and doesn’t create a request.</t>
         </is>
       </c>
       <c r="F66" s="7" t="inlineStr"/>
@@ -39789,7 +39789,7 @@
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>The builder: prices, “urgent”, “maintenance report”</t>
+          <t>The builder: prices, “urgent,” “maintenance report”</t>
         </is>
       </c>
       <c r="F68" s="7" t="inlineStr"/>
@@ -39963,7 +39963,7 @@
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>Rooms, floors and buildings open the same dialog with the same three options: edit, take out of service, delete.</t>
+          <t>Rooms, floors, and buildings open the same dialog with the same three options: edit, take out of service, delete.</t>
         </is>
       </c>
       <c r="F74" s="7" t="inlineStr"/>
@@ -40137,7 +40137,7 @@
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>No — edit it. Number, floor and building can be changed without losing history, stays or work records; everything belongs to the room, not its number. Deleting is for rooms created by mistake without history.</t>
+          <t>No — edit it. Number, floor, and building can be changed without losing history, stays, or work records; everything belongs to the room, not its number. Deleting is for rooms created by mistake without history.</t>
         </is>
       </c>
       <c r="F80" s="7" t="inlineStr"/>
@@ -40572,7 +40572,7 @@
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>The rules apply to everything from the moment you save. Current stays, requests already set and PINs already issued continue unchanged — nothing is converted retroactively.</t>
+          <t>The rules apply to everything from the moment you save. Current stays, requests already set, and PINs already issued continue unchanged — nothing is converted retroactively.</t>
         </is>
       </c>
       <c r="F95" s="7" t="inlineStr"/>
@@ -40717,7 +40717,7 @@
       </c>
       <c r="E100" s="6" t="inlineStr">
         <is>
-          <t>Off by default: rooms are cleaned at the guest’s request and after check-out. That saves water, detergent and working time and is part of the sustainability promise. When it’s on, occupied rooms appear on the board on their own from the day after arrival at the chosen time — except with “Do not disturb”, “No cleaning today”, on the day of departure and if the room has already been cleaned today. If the guest has set a request themselves, their request applies.</t>
+          <t>Off by default: rooms are cleaned at the guest’s request and after check-out. That saves water, detergent, and working time and is part of the sustainability promise. When it’s on, occupied rooms appear on the board on their own from the day after arrival at the chosen time — except with “Do not disturb,” “No cleaning today,” on the day of departure, and if the room has already been cleaned today. If the guest has set a request themselves, their request applies.</t>
         </is>
       </c>
       <c r="F100" s="7" t="inlineStr"/>
@@ -41007,7 +41007,7 @@
       </c>
       <c r="E110" s="6" t="inlineStr">
         <is>
-          <t>If a started cleaning isn’t finished, the room reopens on its own after the time limit, and the history shows “Cleaning not finished (time limit, name)”. The limit should be well above the longest real cleaning — default 90 minutes.</t>
+          <t>If a started cleaning isn’t finished, the room reopens on its own after the time limit, and the history shows “Cleaning not finished (time limit, name).” The limit should be well above the longest real cleaning — default 90 minutes.</t>
         </is>
       </c>
       <c r="F110" s="7" t="inlineStr"/>
@@ -41123,7 +41123,7 @@
       </c>
       <c r="E114" s="6" t="inlineStr">
         <is>
-          <t>Yes. Under “Currency of service prices” you choose the currency in which you enter prices in the service builder; guests, the front desk and the check-out statement then show it that way. Every request remembers its currency, so old requests stay as they were. Existing prices aren’t converted when you switch. You can only switch while no guest is checked in.</t>
+          <t>Yes. Under “Currency of service prices” you choose the currency in which you enter prices in the service builder; guests, the front desk, and the check-out statement then show it that way. Every request remembers its currency, so old requests stay as they were. Existing prices aren’t converted when you switch. You can only switch while no guest is checked in.</t>
         </is>
       </c>
       <c r="F114" s="7" t="inlineStr"/>
@@ -41355,7 +41355,7 @@
       </c>
       <c r="E122" s="6" t="inlineStr">
         <is>
-          <t>PNG, JPG or SVG up to 1 MB. It appears on room sign and check-in sheet at 55 × 16 mm max.; below about 400 px width it looks blurry there. The preview is on a white background — otherwise a light logo meant for dark backgrounds would be invisible on paper. Without a logo, the sheets show the property name.</t>
+          <t>PNG, JPG, or SVG up to 1 MB. It appears on room sign and check-in sheet at 55 × 16 mm max.; below about 400 px width it looks blurry there. The preview is on a white background — otherwise a light logo meant for dark backgrounds would be invisible on paper. Without a logo, the sheets show the property name.</t>
         </is>
       </c>
       <c r="F122" s="7" t="inlineStr"/>
@@ -42225,7 +42225,7 @@
       </c>
       <c r="E152" s="6" t="inlineStr">
         <is>
-          <t>A4 for frames, stands and folders; compact (92 × 130 mm, four per page to cut apart) for door signs and the desk. The choice depends on the occasion and isn’t saved. The QR code is sized for reading distance: 55 mm on A4, 42 mm compact.</t>
+          <t>A4 for frames, stands, and folders; compact (92 × 130 mm, four per page to cut apart) for door signs and the desk. The choice depends on the occasion and isn’t saved. The QR code is sized for reading distance: 55 mm on A4, 42 mm compact.</t>
         </is>
       </c>
       <c r="F152" s="7" t="inlineStr"/>
@@ -42747,7 +42747,7 @@
       </c>
       <c r="E170" s="6" t="inlineStr">
         <is>
-          <t>Housekeeping, front desk, managers — accounts, invitations, access cards, ending and deleting</t>
+          <t>Housekeeping, front desk, managers — accounts, invitations, access cards, ending, and deleting</t>
         </is>
       </c>
       <c r="F170" s="7" t="inlineStr"/>
@@ -43153,7 +43153,7 @@
       </c>
       <c r="E184" s="6" t="inlineStr">
         <is>
-          <t>Almost always, the display name is in the “Username” field. Sign-in uses the short username shown on the access card under “Credentials”. Second cause: the access was ended — then the sign-in page says so.</t>
+          <t>Almost always, the display name is in the “Username” field. Sign-in uses the short username shown on the access card under “Credentials.” Second cause: the access was ended — then the sign-in page says so.</t>
         </is>
       </c>
       <c r="F184" s="7" t="inlineStr"/>
@@ -43269,7 +43269,7 @@
       </c>
       <c r="E188" s="6" t="inlineStr">
         <is>
-          <t>Below the send button you see the delivery status: handed over, delivered or rejected — with the receiving server’s reason. Usually it’s a typo in the address. After a rejection, the address can be unblocked and the email resent; and there’s “Show invitation link” to hand over the link via messenger or on paper. There’s a one-minute wait between two emails to the same person.</t>
+          <t>Below the send button you see the delivery status: handed over, delivered, or rejected — with the receiving server’s reason. Usually it’s a typo in the address. After a rejection, the address can be unblocked and the email resent; and there’s “Show invitation link” to hand over the link via messenger or on paper. There’s a one-minute wait between two emails to the same person.</t>
         </is>
       </c>
       <c r="F188" s="7" t="inlineStr"/>
@@ -43385,7 +43385,7 @@
       </c>
       <c r="E192" s="6" t="inlineStr">
         <is>
-          <t>Front desk: check-in and check-out, priorities, requests, printing check-in sheets, cards and room signs, own password. Not: settings, rooms, services, staff, “Renew code”. Manager: the same rights as the owner within the property, but no access to the account and billing. Only the owner appoints managers.</t>
+          <t>Front desk: check-in and check-out, priorities, requests, printing check-in sheets, cards, and room signs, own password. Not: settings, rooms, services, staff, “Renew code.” Manager: the same rights as the owner within the property, but no access to the account and billing. Only the owner appoints managers.</t>
         </is>
       </c>
       <c r="F192" s="7" t="inlineStr"/>
@@ -43675,7 +43675,7 @@
       </c>
       <c r="E202" s="6" t="inlineStr">
         <is>
-          <t>The service builder: services, options, prices, “urgent”, “maintenance report”</t>
+          <t>The service builder: services, options, prices, “urgent,” “maintenance report”</t>
         </is>
       </c>
       <c r="F202" s="7" t="inlineStr"/>
@@ -44023,7 +44023,7 @@
       </c>
       <c r="E214" s="6" t="inlineStr">
         <is>
-          <t>You create each service in your home language. Below the service, language chips show which guest portal languages it’s already translated into — tapping a language opens the fields for name, description and options, with the source text below each. Feel free to translate with a tool of your choice. If a translation is missing, the guest sees the source text, never an empty field. The front desk always sees requests in the home language. The example services are already translated.</t>
+          <t>You create each service in your home language. Below the service, language chips show which guest portal languages it’s already translated into — tapping a language opens the fields for name, description, and options, with the source text below each. Feel free to translate with a tool of your choice. If a translation is missing, the guest sees the source text, never an empty field. The front desk always sees requests in the home language. The example services are already translated.</t>
         </is>
       </c>
       <c r="F214" s="7" t="inlineStr"/>
@@ -44081,7 +44081,7 @@
       </c>
       <c r="E216" s="6" t="inlineStr">
         <is>
-          <t>No. Name, options and prices are frozen at the time of the request; old requests and statements stay as they were. The “maintenance report” flag, on the other hand, also affects open requests immediately — it decides behavior, not the content of a record.</t>
+          <t>No. Name, options, and prices are frozen at the time of the request; old requests and statements stay as they were. The “maintenance report” flag, on the other hand, also affects open requests immediately — it decides behavior, not the content of a record.</t>
         </is>
       </c>
       <c r="F216" s="7" t="inlineStr"/>
@@ -45444,7 +45444,7 @@
       </c>
       <c r="E263" s="6" t="inlineStr">
         <is>
-          <t>It isn’t blocked, it just has no task: vacant, occupied without a request, “Do not disturb”, no cleaning wanted today (leaf), or a cleaning that applies only later (“from 11:00”). It stays visible so the floor is complete. At the set time, a postponed request switches to open on its own.</t>
+          <t>It isn’t blocked, it just has no task: vacant, occupied without a request, “Do not disturb,” no cleaning wanted today (leaf), or a cleaning that applies only later (“from 11:00”). It stays visible so the floor is complete. At the set time, a postponed request switches to open on its own.</t>
         </is>
       </c>
       <c r="F263" s="7" t="inlineStr"/>
@@ -45502,7 +45502,7 @@
       </c>
       <c r="E265" s="6" t="inlineStr">
         <is>
-          <t>Tap the room without starting: “In 30 min”, “In 1 hr” or “Not today”. “In 30 min” and “In 1 hr” take the room off the board until that time — for the whole team, nobody knocks again in between —, afterwards it’s open again on its own. “Not today” settles the room for today without counting as a cleaning. If the guest still wants cleaning, they tap it in the portal; then it’s open again.</t>
+          <t>Tap the room without starting: “In 30 min,” “In 1 hr” or “Not today.” “In 30 min” and “In 1 hr” take the room off the board until that time — for the whole team, nobody knocks again in between —, afterwards it’s open again on its own. “Not today” settles the room for today without counting as a cleaning. If the guest still wants cleaning, they tap it in the portal; then it’s open again.</t>
         </is>
       </c>
       <c r="F265" s="7" t="inlineStr"/>
@@ -45560,7 +45560,7 @@
       </c>
       <c r="E267" s="6" t="inlineStr">
         <is>
-          <t>After the time limit set by the property (default 90 minutes), the room reopens on its own; the history shows “Cleaning not finished (time limit, name)”. The cleaning then doesn’t count as done in the reports — so the finish slider is always worth it.</t>
+          <t>After the time limit set by the property (default 90 minutes), the room reopens on its own; the history shows “Cleaning not finished (time limit, name).” The cleaning then doesn’t count as done in the reports — so the finish slider is always worth it.</t>
         </is>
       </c>
       <c r="F267" s="7" t="inlineStr"/>
@@ -45850,7 +45850,7 @@
       </c>
       <c r="E277" s="6" t="inlineStr">
         <is>
-          <t>The field contains the display name instead of the short username — that’s on the access card under “Credentials”. Or the access was ended; then the page says so. Scanning the card is the way without typing.</t>
+          <t>The field contains the display name instead of the short username — that’s on the access card under “Credentials.” Or the access was ended; then the page says so. Scanning the card is the way without typing.</t>
         </is>
       </c>
       <c r="F277" s="7" t="inlineStr"/>
@@ -45908,7 +45908,7 @@
       </c>
       <c r="E279" s="6" t="inlineStr">
         <is>
-          <t>From the entries: shift start and end, breaks, other cleaning, start and finish per room. From these, the reports calculate work and cleaning times; the room history shows every cleaning with a name — in team mode as “Housekeeping team”.</t>
+          <t>From the entries: shift start and end, breaks, other cleaning, start and finish per room. From these, the reports calculate work and cleaning times; the room history shows every cleaning with a name — in team mode as “Housekeeping team.”</t>
         </is>
       </c>
       <c r="F279" s="7" t="inlineStr"/>
@@ -46140,7 +46140,7 @@
       </c>
       <c r="E287" s="6" t="inlineStr">
         <is>
-          <t>Access, PIN lock, cleaning and “not before”, Do not disturb, requests, check-out</t>
+          <t>Access, PIN lock, cleaning and “not before,” Do not disturb, requests, check-out</t>
         </is>
       </c>
       <c r="F287" s="7" t="inlineStr"/>
@@ -46256,7 +46256,7 @@
       </c>
       <c r="E291" s="6" t="inlineStr">
         <is>
-          <t>After five wrong PINs, the stay is locked for 15 minutes — even for the correct PIN. This applies only to this room, not to the property. After that it works again; the correct PIN is in the room dialog. Checking out and in again isn’t a good way out: check-out closes open requests and sets the room to “cleaning open”.</t>
+          <t>After five wrong PINs, the stay is locked for 15 minutes — even for the correct PIN. This applies only to this room, not to the property. After that it works again; the correct PIN is in the room dialog. Checking out and in again isn’t a good way out: check-out closes open requests and sets the room to “cleaning open.”</t>
         </is>
       </c>
       <c r="F291" s="7" t="inlineStr"/>
@@ -46372,7 +46372,7 @@
       </c>
       <c r="E295" s="6" t="inlineStr">
         <is>
-          <t>Where the guest stands with cleaning, from the same data as your boards: “planned” (request, priority or daily cleaning due), “from HH:MM” (guest postponed or daily cleaning not yet due), “being cleaned right now”, “cleaned today at HH:MM” or “nothing planned today” — with the reason (day of arrival, day of departure, property cleans on request only). “Cleaned” only counts from this guest’s check-in; a housekeeper’s name never appears. The card updates every 15 seconds.</t>
+          <t>Where the guest stands with cleaning, from the same data as your boards: “planned” (request, priority, or daily cleaning due), “from HH:MM” (guest postponed or daily cleaning not yet due), “being cleaned right now,” “cleaned today at HH:MM” or “nothing planned today” — with the reason (day of arrival, day of departure, property cleans on request only). “Cleaned” only counts from this guest’s check-in; a housekeeper’s name never appears. The card updates every 15 seconds.</t>
         </is>
       </c>
       <c r="F295" s="7" t="inlineStr"/>
@@ -46546,7 +46546,7 @@
       </c>
       <c r="E301" s="6" t="inlineStr">
         <is>
-          <t>No. They see prices for information and order with one tap; the request lands with you under “Requests”. At check-out, RoSe shows the total of what was provided — payment is collected at the desk as before.</t>
+          <t>No. They see prices for information and order with one tap; the request lands with you under “Requests.” At check-out, RoSe shows the total of what was provided — payment is collected at the desk as before.</t>
         </is>
       </c>
       <c r="F301" s="7" t="inlineStr"/>
@@ -46662,7 +46662,7 @@
       </c>
       <c r="E305" s="6" t="inlineStr">
         <is>
-          <t>Nothing. A stay is a room, a period, a PIN or a link — no name, no address. An address entered for the access email isn’t stored. At check-out, PIN, link and sign-in expire.</t>
+          <t>Nothing. A stay is a room, a period, a PIN, or a link — no name, no address. An address entered for the access email isn’t stored. At check-out, PIN, link, and sign-in expire.</t>
         </is>
       </c>
       <c r="F305" s="7" t="inlineStr"/>
@@ -46836,7 +46836,7 @@
       </c>
       <c r="E311" s="6" t="inlineStr">
         <is>
-          <t>Work, break and cleaning times from the entries, irregularities, demand by hour</t>
+          <t>Work, break, and cleaning times from the entries, irregularities, demand by hour</t>
         </is>
       </c>
       <c r="F311" s="7" t="inlineStr"/>
@@ -47445,7 +47445,7 @@
       </c>
       <c r="E332" s="6" t="inlineStr">
         <is>
-          <t>Sign-in address, display name and password of the signed-in person</t>
+          <t>Sign-in address, display name, and password of the signed-in person</t>
         </is>
       </c>
       <c r="F332" s="7" t="inlineStr"/>
@@ -47677,7 +47677,7 @@
       </c>
       <c r="E340" s="6" t="inlineStr">
         <is>
-          <t>Yes, here under “Change sign-in address” — for owners, managers and front desk. You enter your current password and the new address; a confirmation link goes to the new address, and only clicking it makes the switch. Until then, you keep signing in with the old address. After the switch, the old address receives a notice.</t>
+          <t>Yes, here under “Change sign-in address” — for owners, managers, and front desk. You enter your current password and the new address; a confirmation link goes to the new address, and only clicking it makes the switch. Until then, you keep signing in with the old address. After the switch, the old address receives a notice.</t>
         </is>
       </c>
       <c r="F340" s="7" t="inlineStr"/>
@@ -47967,7 +47967,7 @@
       </c>
       <c r="E350" s="6" t="inlineStr">
         <is>
-          <t>The properties page is the entry point for owners and managers: all accessible properties with their status (open cleanings, requests), and below, for the owner, the account box and “Add property”. The front desk never sees this page — it knows exactly one property.</t>
+          <t>The properties page is the entry point for owners and managers: all accessible properties with their status (open cleanings, requests), and below, for the owner, the account box and “Add property.” The front desk never sees this page — it knows exactly one property.</t>
         </is>
       </c>
       <c r="F350" s="7" t="inlineStr"/>
@@ -48141,7 +48141,7 @@
       </c>
       <c r="E356" s="6" t="inlineStr">
         <is>
-          <t>Completely removing a property or the whole account — with a preview in figures and the name typed to confirm; it can’t be undone. Unlike day-to-day work, where records deliberately survive, it clears everything: history, sign-in accounts and logo too. Only the invoice records remain, because they have to be kept. Deleting the account is also the cancellation at the end of the month: for the current month, a final invoice is created on deletion, and the dialog shows the amount beforehand (nothing in the free month).</t>
+          <t>Completely removing a property or the whole account — with a preview in figures and the name typed to confirm; it can’t be undone. Unlike day-to-day work, where records deliberately survive, it clears everything: history, sign-in accounts, and logo too. Only the invoice records remain, because they have to be kept. Deleting the account is also the cancellation at the end of the month: for the current month, a final invoice is created on deletion, and the dialog shows the amount beforehand (nothing in the free month).</t>
         </is>
       </c>
       <c r="F356" s="7" t="inlineStr"/>
@@ -48199,7 +48199,7 @@
       </c>
       <c r="E358" s="6" t="inlineStr">
         <is>
-          <t>It’s created with its own address, rooms, staff and rules. Billing is per room across all properties of the account; the minimum amount applies per account, not per property.</t>
+          <t>It’s created with its own address, rooms, staff, and rules. Billing is per room across all properties of the account; the minimum amount applies per account, not per property.</t>
         </is>
       </c>
       <c r="F358" s="7" t="inlineStr"/>
@@ -49330,7 +49330,7 @@
       </c>
       <c r="E397" s="6" t="inlineStr">
         <is>
-          <t>Housekeeping, front desk and managers — create, end access, print access cards</t>
+          <t>Housekeeping, front desk, and managers — create, end access, print access cards</t>
         </is>
       </c>
       <c r="F397" s="7" t="inlineStr"/>
@@ -49504,7 +49504,7 @@
       </c>
       <c r="E403" s="6" t="inlineStr">
         <is>
-          <t>Replica: the guest portal on a phone — cleaning, “not before”, skipping, Do not disturb, services</t>
+          <t>Replica: the guest portal on a phone — cleaning, “not before,” skipping, Do not disturb, services</t>
         </is>
       </c>
       <c r="F403" s="7" t="inlineStr"/>
@@ -49562,7 +49562,7 @@
       </c>
       <c r="E405" s="6" t="inlineStr">
         <is>
-          <t>Work times from the entries, irregularities and when guests want cleaning</t>
+          <t>Work times from the entries, irregularities, and when guests want cleaning</t>
         </is>
       </c>
       <c r="F405" s="7" t="inlineStr"/>
@@ -49620,7 +49620,7 @@
       </c>
       <c r="E407" s="6" t="inlineStr">
         <is>
-          <t>What the account costs, how rooms are counted and where payment method and invoices are</t>
+          <t>What the account costs, how rooms are counted, and where payment method and invoices are</t>
         </is>
       </c>
       <c r="F407" s="7" t="inlineStr"/>
@@ -54027,7 +54027,7 @@
       </c>
       <c r="E582" s="6" t="inlineStr">
         <is>
-          <t>Time zone set — daily cleaning, check-out time and reports calculate correctly</t>
+          <t>Time zone set — daily cleaning, check-out time, and reports calculate correctly</t>
         </is>
       </c>
       <c r="F582" s="7" t="inlineStr"/>
@@ -58474,7 +58474,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Towels, repairs and more — the front desk sees it right away.</t>
+          <t>Towels, repairs, and more — the front desk sees it right away.</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr"/>

</xml_diff>